<commit_message>
Calculate price levels automatically
</commit_message>
<xml_diff>
--- a/public/modelos/lista-precos-exemplo.xlsx
+++ b/public/modelos/lista-precos-exemplo.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista de Preços" sheetId="1" r:id="R905b78147cb14101"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="2" r:id="Rf7c0a60edccf4f54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista de Preços" sheetId="1" r:id="Rcfea1d35f1094db6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="2" r:id="R9c25b7d3e6dc4d19"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -446,154 +446,154 @@
         <x:v>Cliente Final BA</x:v>
       </x:c>
       <x:c r="J1" s="13" t="str">
-        <x:v>Cliente N2 BA</x:v>
+        <x:v>Cliente Nível 2 BA</x:v>
       </x:c>
       <x:c r="K1" s="13" t="str">
-        <x:v>Cliente N3 BA</x:v>
+        <x:v>Cliente Nível 3 BA</x:v>
       </x:c>
       <x:c r="L1" s="13" t="str">
         <x:v>Cliente Final MA</x:v>
       </x:c>
       <x:c r="M1" s="13" t="str">
-        <x:v>Cliente N2 MA</x:v>
+        <x:v>Cliente Nível 2 MA</x:v>
       </x:c>
       <x:c r="N1" s="13" t="str">
-        <x:v>Cliente N3 MA</x:v>
+        <x:v>Cliente Nível 3 MA</x:v>
       </x:c>
       <x:c r="O1" s="13" t="str">
         <x:v>Cliente Final PI</x:v>
       </x:c>
       <x:c r="P1" s="13" t="str">
-        <x:v>Cliente N2 PI</x:v>
+        <x:v>Cliente Nível 2 PI</x:v>
       </x:c>
       <x:c r="Q1" s="13" t="str">
-        <x:v>Cliente N3 PI</x:v>
+        <x:v>Cliente Nível 3 PI</x:v>
       </x:c>
       <x:c r="R1" s="13" t="str">
         <x:v>Cliente Final TO</x:v>
       </x:c>
       <x:c r="S1" s="13" t="str">
-        <x:v>Cliente N2 TO</x:v>
+        <x:v>Cliente Nível 2 TO</x:v>
       </x:c>
       <x:c r="T1" s="13" t="str">
-        <x:v>Cliente N3 TO</x:v>
+        <x:v>Cliente Nível 3 TO</x:v>
       </x:c>
       <x:c r="U1" s="13" t="str">
         <x:v>Cliente Final RS</x:v>
       </x:c>
       <x:c r="V1" s="13" t="str">
-        <x:v>Cliente N2 RS</x:v>
+        <x:v>Cliente Nível 2 RS</x:v>
       </x:c>
       <x:c r="W1" s="13" t="str">
-        <x:v>Cliente N3 RS</x:v>
+        <x:v>Cliente Nível 3 RS</x:v>
       </x:c>
       <x:c r="X1" s="13" t="str">
         <x:v>Cliente Final SC</x:v>
       </x:c>
       <x:c r="Y1" s="13" t="str">
-        <x:v>Cliente N2 SC</x:v>
+        <x:v>Cliente Nível 2 SC</x:v>
       </x:c>
       <x:c r="Z1" s="13" t="str">
-        <x:v>Cliente N3 SC</x:v>
+        <x:v>Cliente Nível 3 SC</x:v>
       </x:c>
       <x:c r="AA1" s="13" t="str">
         <x:v>Cliente Final PR</x:v>
       </x:c>
       <x:c r="AB1" s="13" t="str">
-        <x:v>Cliente N2 PR</x:v>
+        <x:v>Cliente Nível 2 PR</x:v>
       </x:c>
       <x:c r="AC1" s="13" t="str">
-        <x:v>Cliente N3 PR</x:v>
+        <x:v>Cliente Nível 3 PR</x:v>
       </x:c>
       <x:c r="AD1" s="13" t="str">
         <x:v>Cliente Final SP</x:v>
       </x:c>
       <x:c r="AE1" s="13" t="str">
-        <x:v>Cliente N2 SP</x:v>
+        <x:v>Cliente Nível 2 SP</x:v>
       </x:c>
       <x:c r="AF1" s="13" t="str">
-        <x:v>Cliente N3 SP</x:v>
+        <x:v>Cliente Nível 3 SP</x:v>
       </x:c>
       <x:c r="AG1" s="13" t="str">
         <x:v>Cliente Final MG</x:v>
       </x:c>
       <x:c r="AH1" s="13" t="str">
-        <x:v>Cliente N2 MG</x:v>
+        <x:v>Cliente Nível 2 MG</x:v>
       </x:c>
       <x:c r="AI1" s="13" t="str">
-        <x:v>Cliente N3 MG</x:v>
+        <x:v>Cliente Nível 3 MG</x:v>
       </x:c>
       <x:c r="AJ1" s="13" t="str">
         <x:v>Cliente Final MS</x:v>
       </x:c>
       <x:c r="AK1" s="13" t="str">
-        <x:v>Cliente N2 MS</x:v>
+        <x:v>Cliente Nível 2 MS</x:v>
       </x:c>
       <x:c r="AL1" s="13" t="str">
-        <x:v>Cliente N3 MS</x:v>
+        <x:v>Cliente Nível 3 MS</x:v>
       </x:c>
       <x:c r="AM1" s="13" t="str">
         <x:v>Cliente Final MT</x:v>
       </x:c>
       <x:c r="AN1" s="13" t="str">
-        <x:v>Cliente N2 MT</x:v>
+        <x:v>Cliente Nível 2 MT</x:v>
       </x:c>
       <x:c r="AO1" s="13" t="str">
-        <x:v>Cliente N3 MT</x:v>
+        <x:v>Cliente Nível 3 MT</x:v>
       </x:c>
       <x:c r="AP1" s="13" t="str">
         <x:v>Cliente Final DF</x:v>
       </x:c>
       <x:c r="AQ1" s="13" t="str">
-        <x:v>Cliente N2 DF</x:v>
+        <x:v>Cliente Nível 2 DF</x:v>
       </x:c>
       <x:c r="AR1" s="13" t="str">
-        <x:v>Cliente N3 DF</x:v>
+        <x:v>Cliente Nível 3 DF</x:v>
       </x:c>
       <x:c r="AS1" s="13" t="str">
         <x:v>Cliente Final RR</x:v>
       </x:c>
       <x:c r="AT1" s="13" t="str">
-        <x:v>Cliente N2 RR</x:v>
+        <x:v>Cliente Nível 2 RR</x:v>
       </x:c>
       <x:c r="AU1" s="13" t="str">
-        <x:v>Cliente N3 RR</x:v>
+        <x:v>Cliente Nível 3 RR</x:v>
       </x:c>
       <x:c r="AV1" s="13" t="str">
         <x:v>Cliente Final PA</x:v>
       </x:c>
       <x:c r="AW1" s="13" t="str">
-        <x:v>Cliente N2 PA</x:v>
+        <x:v>Cliente Nível 2 PA</x:v>
       </x:c>
       <x:c r="AX1" s="13" t="str">
-        <x:v>Cliente N3 PA</x:v>
+        <x:v>Cliente Nível 3 PA</x:v>
       </x:c>
       <x:c r="AY1" s="13" t="str">
         <x:v>Cliente Final GO</x:v>
       </x:c>
       <x:c r="AZ1" s="13" t="str">
-        <x:v>Cliente N2 GO</x:v>
+        <x:v>Cliente Nível 2 GO</x:v>
       </x:c>
       <x:c r="BA1" s="13" t="str">
-        <x:v>Cliente N3 GO</x:v>
+        <x:v>Cliente Nível 3 GO</x:v>
       </x:c>
       <x:c r="BB1" s="13" t="str">
         <x:v>Cliente Final PY</x:v>
       </x:c>
       <x:c r="BC1" s="13" t="str">
-        <x:v>Cliente N2 PY</x:v>
+        <x:v>Cliente Nível 2 PY</x:v>
       </x:c>
       <x:c r="BD1" s="13" t="str">
-        <x:v>Cliente N3 PY</x:v>
+        <x:v>Cliente Nível 3 PY</x:v>
       </x:c>
       <x:c r="BE1" s="13" t="str">
         <x:v>Cliente Final RO</x:v>
       </x:c>
       <x:c r="BF1" s="13" t="str">
-        <x:v>Cliente N2 RO</x:v>
+        <x:v>Cliente Nível 2 RO</x:v>
       </x:c>
       <x:c r="BG1" s="13" t="str">
-        <x:v>Cliente N3 RO</x:v>
+        <x:v>Cliente Nível 3 RO</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
@@ -622,62 +622,128 @@
         <x:v>1250.5</x:v>
       </x:c>
       <x:c r="I2" s="15"/>
-      <x:c r="J2" s="15"/>
-      <x:c r="K2" s="15"/>
+      <x:c r="J2" s="15" t="str">
+        <x:f>IF(I2="","",I2*0.9)</x:f>
+      </x:c>
+      <x:c r="K2" s="15" t="str">
+        <x:f>IF(I2="","",I2*0.8)</x:f>
+      </x:c>
       <x:c r="L2" s="15"/>
-      <x:c r="M2" s="15"/>
-      <x:c r="N2" s="15"/>
+      <x:c r="M2" s="15" t="str">
+        <x:f>IF(L2="","",L2*0.9)</x:f>
+      </x:c>
+      <x:c r="N2" s="15" t="str">
+        <x:f>IF(L2="","",L2*0.8)</x:f>
+      </x:c>
       <x:c r="O2" s="15"/>
-      <x:c r="P2" s="15"/>
-      <x:c r="Q2" s="15"/>
+      <x:c r="P2" s="15" t="str">
+        <x:f>IF(O2="","",O2*0.9)</x:f>
+      </x:c>
+      <x:c r="Q2" s="15" t="str">
+        <x:f>IF(O2="","",O2*0.8)</x:f>
+      </x:c>
       <x:c r="R2" s="15"/>
-      <x:c r="S2" s="15"/>
-      <x:c r="T2" s="15"/>
+      <x:c r="S2" s="15" t="str">
+        <x:f>IF(R2="","",R2*0.9)</x:f>
+      </x:c>
+      <x:c r="T2" s="15" t="str">
+        <x:f>IF(R2="","",R2*0.8)</x:f>
+      </x:c>
       <x:c r="U2" s="15"/>
-      <x:c r="V2" s="15"/>
-      <x:c r="W2" s="15"/>
+      <x:c r="V2" s="15" t="str">
+        <x:f>IF(U2="","",U2*0.9)</x:f>
+      </x:c>
+      <x:c r="W2" s="15" t="str">
+        <x:f>IF(U2="","",U2*0.8)</x:f>
+      </x:c>
       <x:c r="X2" s="15"/>
-      <x:c r="Y2" s="15"/>
-      <x:c r="Z2" s="15"/>
+      <x:c r="Y2" s="15" t="str">
+        <x:f>IF(X2="","",X2*0.9)</x:f>
+      </x:c>
+      <x:c r="Z2" s="15" t="str">
+        <x:f>IF(X2="","",X2*0.8)</x:f>
+      </x:c>
       <x:c r="AA2" s="15"/>
-      <x:c r="AB2" s="15"/>
-      <x:c r="AC2" s="15"/>
+      <x:c r="AB2" s="15" t="str">
+        <x:f>IF(AA2="","",AA2*0.9)</x:f>
+      </x:c>
+      <x:c r="AC2" s="15" t="str">
+        <x:f>IF(AA2="","",AA2*0.8)</x:f>
+      </x:c>
       <x:c r="AD2" s="15" t="n">
         <x:v>1750</x:v>
       </x:c>
       <x:c r="AE2" s="15" t="n">
-        <x:v>1600</x:v>
+        <x:f>IF(AD2="","",AD2*0.9)</x:f>
+        <x:v>1575</x:v>
       </x:c>
       <x:c r="AF2" s="15" t="n">
-        <x:v>1450</x:v>
+        <x:f>IF(AD2="","",AD2*0.8)</x:f>
+        <x:v>1400</x:v>
       </x:c>
       <x:c r="AG2" s="15"/>
-      <x:c r="AH2" s="15"/>
-      <x:c r="AI2" s="15"/>
+      <x:c r="AH2" s="15" t="str">
+        <x:f>IF(AG2="","",AG2*0.9)</x:f>
+      </x:c>
+      <x:c r="AI2" s="15" t="str">
+        <x:f>IF(AG2="","",AG2*0.8)</x:f>
+      </x:c>
       <x:c r="AJ2" s="15"/>
-      <x:c r="AK2" s="15"/>
-      <x:c r="AL2" s="15"/>
+      <x:c r="AK2" s="15" t="str">
+        <x:f>IF(AJ2="","",AJ2*0.9)</x:f>
+      </x:c>
+      <x:c r="AL2" s="15" t="str">
+        <x:f>IF(AJ2="","",AJ2*0.8)</x:f>
+      </x:c>
       <x:c r="AM2" s="15"/>
-      <x:c r="AN2" s="15"/>
-      <x:c r="AO2" s="15"/>
+      <x:c r="AN2" s="15" t="str">
+        <x:f>IF(AM2="","",AM2*0.9)</x:f>
+      </x:c>
+      <x:c r="AO2" s="15" t="str">
+        <x:f>IF(AM2="","",AM2*0.8)</x:f>
+      </x:c>
       <x:c r="AP2" s="15"/>
-      <x:c r="AQ2" s="15"/>
-      <x:c r="AR2" s="15"/>
+      <x:c r="AQ2" s="15" t="str">
+        <x:f>IF(AP2="","",AP2*0.9)</x:f>
+      </x:c>
+      <x:c r="AR2" s="15" t="str">
+        <x:f>IF(AP2="","",AP2*0.8)</x:f>
+      </x:c>
       <x:c r="AS2" s="15"/>
-      <x:c r="AT2" s="15"/>
-      <x:c r="AU2" s="15"/>
+      <x:c r="AT2" s="15" t="str">
+        <x:f>IF(AS2="","",AS2*0.9)</x:f>
+      </x:c>
+      <x:c r="AU2" s="15" t="str">
+        <x:f>IF(AS2="","",AS2*0.8)</x:f>
+      </x:c>
       <x:c r="AV2" s="15"/>
-      <x:c r="AW2" s="15"/>
-      <x:c r="AX2" s="15"/>
+      <x:c r="AW2" s="15" t="str">
+        <x:f>IF(AV2="","",AV2*0.9)</x:f>
+      </x:c>
+      <x:c r="AX2" s="15" t="str">
+        <x:f>IF(AV2="","",AV2*0.8)</x:f>
+      </x:c>
       <x:c r="AY2" s="15"/>
-      <x:c r="AZ2" s="15"/>
-      <x:c r="BA2" s="15"/>
+      <x:c r="AZ2" s="15" t="str">
+        <x:f>IF(AY2="","",AY2*0.9)</x:f>
+      </x:c>
+      <x:c r="BA2" s="15" t="str">
+        <x:f>IF(AY2="","",AY2*0.8)</x:f>
+      </x:c>
       <x:c r="BB2" s="15"/>
-      <x:c r="BC2" s="15"/>
-      <x:c r="BD2" s="15"/>
+      <x:c r="BC2" s="15" t="str">
+        <x:f>IF(BB2="","",BB2*0.9)</x:f>
+      </x:c>
+      <x:c r="BD2" s="15" t="str">
+        <x:f>IF(BB2="","",BB2*0.8)</x:f>
+      </x:c>
       <x:c r="BE2" s="15"/>
-      <x:c r="BF2" s="15"/>
-      <x:c r="BG2" s="15"/>
+      <x:c r="BF2" s="15" t="str">
+        <x:f>IF(BE2="","",BE2*0.9)</x:f>
+      </x:c>
+      <x:c r="BG2" s="15" t="str">
+        <x:f>IF(BE2="","",BE2*0.8)</x:f>
+      </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
       <x:c r="A3" s="14" t="str">
@@ -705,62 +771,128 @@
         <x:v>980</x:v>
       </x:c>
       <x:c r="I3" s="15"/>
-      <x:c r="J3" s="15"/>
-      <x:c r="K3" s="15"/>
+      <x:c r="J3" s="15" t="str">
+        <x:f>IF(I3="","",I3*0.9)</x:f>
+      </x:c>
+      <x:c r="K3" s="15" t="str">
+        <x:f>IF(I3="","",I3*0.8)</x:f>
+      </x:c>
       <x:c r="L3" s="15"/>
-      <x:c r="M3" s="15"/>
-      <x:c r="N3" s="15"/>
+      <x:c r="M3" s="15" t="str">
+        <x:f>IF(L3="","",L3*0.9)</x:f>
+      </x:c>
+      <x:c r="N3" s="15" t="str">
+        <x:f>IF(L3="","",L3*0.8)</x:f>
+      </x:c>
       <x:c r="O3" s="15"/>
-      <x:c r="P3" s="15"/>
-      <x:c r="Q3" s="15"/>
+      <x:c r="P3" s="15" t="str">
+        <x:f>IF(O3="","",O3*0.9)</x:f>
+      </x:c>
+      <x:c r="Q3" s="15" t="str">
+        <x:f>IF(O3="","",O3*0.8)</x:f>
+      </x:c>
       <x:c r="R3" s="15"/>
-      <x:c r="S3" s="15"/>
-      <x:c r="T3" s="15"/>
+      <x:c r="S3" s="15" t="str">
+        <x:f>IF(R3="","",R3*0.9)</x:f>
+      </x:c>
+      <x:c r="T3" s="15" t="str">
+        <x:f>IF(R3="","",R3*0.8)</x:f>
+      </x:c>
       <x:c r="U3" s="15"/>
-      <x:c r="V3" s="15"/>
-      <x:c r="W3" s="15"/>
+      <x:c r="V3" s="15" t="str">
+        <x:f>IF(U3="","",U3*0.9)</x:f>
+      </x:c>
+      <x:c r="W3" s="15" t="str">
+        <x:f>IF(U3="","",U3*0.8)</x:f>
+      </x:c>
       <x:c r="X3" s="15"/>
-      <x:c r="Y3" s="15"/>
-      <x:c r="Z3" s="15"/>
+      <x:c r="Y3" s="15" t="str">
+        <x:f>IF(X3="","",X3*0.9)</x:f>
+      </x:c>
+      <x:c r="Z3" s="15" t="str">
+        <x:f>IF(X3="","",X3*0.8)</x:f>
+      </x:c>
       <x:c r="AA3" s="15"/>
-      <x:c r="AB3" s="15"/>
-      <x:c r="AC3" s="15"/>
+      <x:c r="AB3" s="15" t="str">
+        <x:f>IF(AA3="","",AA3*0.9)</x:f>
+      </x:c>
+      <x:c r="AC3" s="15" t="str">
+        <x:f>IF(AA3="","",AA3*0.8)</x:f>
+      </x:c>
       <x:c r="AD3" s="15" t="n">
         <x:v>1750</x:v>
       </x:c>
       <x:c r="AE3" s="15" t="n">
-        <x:v>1600</x:v>
+        <x:f>IF(AD3="","",AD3*0.9)</x:f>
+        <x:v>1575</x:v>
       </x:c>
       <x:c r="AF3" s="15" t="n">
-        <x:v>1450</x:v>
+        <x:f>IF(AD3="","",AD3*0.8)</x:f>
+        <x:v>1400</x:v>
       </x:c>
       <x:c r="AG3" s="15"/>
-      <x:c r="AH3" s="15"/>
-      <x:c r="AI3" s="15"/>
+      <x:c r="AH3" s="15" t="str">
+        <x:f>IF(AG3="","",AG3*0.9)</x:f>
+      </x:c>
+      <x:c r="AI3" s="15" t="str">
+        <x:f>IF(AG3="","",AG3*0.8)</x:f>
+      </x:c>
       <x:c r="AJ3" s="15"/>
-      <x:c r="AK3" s="15"/>
-      <x:c r="AL3" s="15"/>
+      <x:c r="AK3" s="15" t="str">
+        <x:f>IF(AJ3="","",AJ3*0.9)</x:f>
+      </x:c>
+      <x:c r="AL3" s="15" t="str">
+        <x:f>IF(AJ3="","",AJ3*0.8)</x:f>
+      </x:c>
       <x:c r="AM3" s="15"/>
-      <x:c r="AN3" s="15"/>
-      <x:c r="AO3" s="15"/>
+      <x:c r="AN3" s="15" t="str">
+        <x:f>IF(AM3="","",AM3*0.9)</x:f>
+      </x:c>
+      <x:c r="AO3" s="15" t="str">
+        <x:f>IF(AM3="","",AM3*0.8)</x:f>
+      </x:c>
       <x:c r="AP3" s="15"/>
-      <x:c r="AQ3" s="15"/>
-      <x:c r="AR3" s="15"/>
+      <x:c r="AQ3" s="15" t="str">
+        <x:f>IF(AP3="","",AP3*0.9)</x:f>
+      </x:c>
+      <x:c r="AR3" s="15" t="str">
+        <x:f>IF(AP3="","",AP3*0.8)</x:f>
+      </x:c>
       <x:c r="AS3" s="15"/>
-      <x:c r="AT3" s="15"/>
-      <x:c r="AU3" s="15"/>
+      <x:c r="AT3" s="15" t="str">
+        <x:f>IF(AS3="","",AS3*0.9)</x:f>
+      </x:c>
+      <x:c r="AU3" s="15" t="str">
+        <x:f>IF(AS3="","",AS3*0.8)</x:f>
+      </x:c>
       <x:c r="AV3" s="15"/>
-      <x:c r="AW3" s="15"/>
-      <x:c r="AX3" s="15"/>
+      <x:c r="AW3" s="15" t="str">
+        <x:f>IF(AV3="","",AV3*0.9)</x:f>
+      </x:c>
+      <x:c r="AX3" s="15" t="str">
+        <x:f>IF(AV3="","",AV3*0.8)</x:f>
+      </x:c>
       <x:c r="AY3" s="15"/>
-      <x:c r="AZ3" s="15"/>
-      <x:c r="BA3" s="15"/>
+      <x:c r="AZ3" s="15" t="str">
+        <x:f>IF(AY3="","",AY3*0.9)</x:f>
+      </x:c>
+      <x:c r="BA3" s="15" t="str">
+        <x:f>IF(AY3="","",AY3*0.8)</x:f>
+      </x:c>
       <x:c r="BB3" s="15"/>
-      <x:c r="BC3" s="15"/>
-      <x:c r="BD3" s="15"/>
+      <x:c r="BC3" s="15" t="str">
+        <x:f>IF(BB3="","",BB3*0.9)</x:f>
+      </x:c>
+      <x:c r="BD3" s="15" t="str">
+        <x:f>IF(BB3="","",BB3*0.8)</x:f>
+      </x:c>
       <x:c r="BE3" s="15"/>
-      <x:c r="BF3" s="15"/>
-      <x:c r="BG3" s="15"/>
+      <x:c r="BF3" s="15" t="str">
+        <x:f>IF(BE3="","",BE3*0.9)</x:f>
+      </x:c>
+      <x:c r="BG3" s="15" t="str">
+        <x:f>IF(BE3="","",BE3*0.8)</x:f>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -818,7 +950,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="22" t="str">
-        <x:v>Preencha o preço Netprice 26 e, quando aplicável, os preços por UF para Cliente Final, N2 e N3.</x:v>
+        <x:v>Preencha uma linha por PN e informe apenas o Netprice 26 e os preços Cliente final por UF. Cliente nível 2 e Cliente nível 3 são calculados automaticamente.</x:v>
       </x:c>
       <x:c r="C4" s="22"/>
       <x:c r="D4" s="24"/>
@@ -879,7 +1011,7 @@
         <x:v>Blocos por UF</x:v>
       </x:c>
       <x:c r="C9" s="22" t="str">
-        <x:v>Cliente Final UF · Cliente N2 UF · Cliente N3 UF</x:v>
+        <x:v>Cliente final UF · Cliente nível 2 UF (90%) · Cliente nível 3 UF (80%)</x:v>
       </x:c>
       <x:c r="D9" s="24"/>
       <x:c r="E9" s="24"/>
@@ -891,7 +1023,7 @@
         <x:v>Exemplo preenchido</x:v>
       </x:c>
       <x:c r="C10" s="22" t="str">
-        <x:v>Os valores demonstrativos estão apenas em SP para facilitar a conferência.</x:v>
+        <x:v>Os valores demonstrativos estão apenas em SP; os níveis 2 e 3 usam fórmulas sobre o Cliente final.</x:v>
       </x:c>
       <x:c r="D10" s="24"/>
       <x:c r="E10" s="24"/>

</xml_diff>